<commit_message>
deploy: main → 68e41dd6b959675cc022bafe1a455b8c90f88677
</commit_message>
<xml_diff>
--- a/StructureDefinition-IneraPatient.xlsx
+++ b/StructureDefinition-IneraPatient.xlsx
@@ -27,7 +27,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://fhir.inera.se/ig/template/StructureDefinition/IneraPatient</t>
+    <t>https://pub.regionstockholm.se/fhir/StructureDefinition/Testmall/StructureDefinition/IneraPatient</t>
   </si>
   <si>
     <t>Identifier</t>
@@ -69,13 +69,13 @@
     <t>Publisher</t>
   </si>
   <si>
-    <t>Inera AB</t>
+    <t>Region Stockholm</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>Inera AB (https://www.inera.se)</t>
+    <t>Region Stockholm (https://www.regionstockholm.se)</t>
   </si>
   <si>
     <t>Jurisdiction</t>

</xml_diff>